<commit_message>
Completely redid the Logging to use real logging.
</commit_message>
<xml_diff>
--- a/Test/OrthoMill1.xlsx
+++ b/Test/OrthoMill1.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JTWhitney\PycharmProjects\ScheduleDateRefresher\Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F277533C-B765-484A-8D91-FCA8945CDA0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A89BAA9-20C5-448C-B35D-A98A9F55847C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31260" yWindow="675" windowWidth="21600" windowHeight="11385" tabRatio="206" xr2:uid="{7D91035E-7C02-4707-AA65-6CEC655CC548}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="206" xr2:uid="{7D91035E-7C02-4707-AA65-6CEC655CC548}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Schedule" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateCount="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>